<commit_message>
Agrega la estrategia de respuesta y el tipo de control (Bow-Tie) a la matriz de riesgos
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_matriz_riesgos.xlsx
+++ b/plantillas/plantilla_matriz_riesgos.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -567,6 +567,13 @@
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>7. Las filas grises son el ejemplo de FarmApp de la guía (Paso 3): bórrelas antes de entregar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>8. Cada riesgo lleva una Estrategia de respuesta (Eliminar / Reducir / Transferir / Aceptar) y el tipo de Control de su mitigación (Preventivo: actúa antes del evento y evita que ocurra; Reactivo: actúa después y reduce el daño). Al menos un riesgo debe quedar con estrategia Aceptar y su justificación escrita en la misma celda: aceptar sin decirlo es no haber mirado.</t>
         </is>
       </c>
     </row>
@@ -581,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -593,8 +600,10 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -645,10 +654,20 @@
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
+          <t>Estrategia (Eliminar / Reducir / Transferir / Aceptar)</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Control (Preventivo / Reactivo)</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
           <t>Prioridad</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Fase del plan que lo mitiga</t>
         </is>
@@ -699,10 +718,20 @@
           <t>Sincronización casi en tiempo real (CDC)</t>
         </is>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Reducir</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>Preventivo</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Mediano plazo</t>
         </is>
@@ -753,10 +782,20 @@
           <t>Reconciliación automática con alertas y trazabilidad</t>
         </is>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Reducir</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Reactivo</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Mediano plazo</t>
         </is>
@@ -807,10 +846,20 @@
           <t>TLS en todos los subdominios y cifrado de datos de pago en tránsito</t>
         </is>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Reducir</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Preventivo</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Corto plazo</t>
         </is>
@@ -861,10 +910,20 @@
           <t>Consentimiento explícito</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Eliminar</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Preventivo</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Quick win</t>
         </is>
@@ -915,10 +974,20 @@
           <t>Proveedor alterno con SLA de respaldo</t>
         </is>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Transferir</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Reactivo</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Gobernanza / cambios</t>
         </is>
@@ -969,30 +1038,88 @@
           <t>Redundancia del balanceador de carga</t>
         </is>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Reducir</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Preventivo</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Largo plazo</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="7">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Reportes internos de ventas lentos en cierre de mes</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Los reportes consultan la misma base de datos transaccional del POS</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Taller 4</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H8" s="5">
         <f>IF(OR(F8="",G8=""),"",MATCH(F8,{"Bajo","Medio","Alto","Crítico"},0)*MATCH(G8,{"Baja","Media","Alta"},0))</f>
         <v/>
       </c>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="n"/>
-      <c r="K8" s="6" t="n"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Ninguna por ahora: se monitorea el tiempo de respuesta y se revisa si supera 30 s</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Aceptar (Nivel 1, componente secundario: una réplica de lectura cuesta más que el daño esperado)</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Reactivo</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>Gobernanza / cambios</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -1009,6 +1136,8 @@
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="n"/>
+      <c r="M9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -1025,6 +1154,8 @@
       <c r="I10" s="6" t="n"/>
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -1041,6 +1172,8 @@
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
+      <c r="M11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
@@ -1057,6 +1190,8 @@
       <c r="I12" s="6" t="n"/>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+      <c r="M12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -1073,6 +1208,8 @@
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+      <c r="M13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -1089,6 +1226,8 @@
       <c r="I14" s="6" t="n"/>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+      <c r="M14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -1105,6 +1244,8 @@
       <c r="I15" s="6" t="n"/>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
+      <c r="M15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
@@ -1121,6 +1262,8 @@
       <c r="I16" s="6" t="n"/>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n"/>
+      <c r="M16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
@@ -1137,6 +1280,8 @@
       <c r="I17" s="6" t="n"/>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="M17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -1153,6 +1298,8 @@
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
+      <c r="M18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
@@ -1169,6 +1316,8 @@
       <c r="I19" s="6" t="n"/>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+      <c r="M19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
@@ -1185,6 +1334,8 @@
       <c r="I20" s="6" t="n"/>
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+      <c r="M20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
@@ -1201,6 +1352,8 @@
       <c r="I21" s="6" t="n"/>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
+      <c r="M21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
@@ -1217,6 +1370,8 @@
       <c r="I22" s="6" t="n"/>
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+      <c r="M22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
@@ -1233,6 +1388,8 @@
       <c r="I23" s="6" t="n"/>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
+      <c r="M23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
@@ -1249,6 +1406,8 @@
       <c r="I24" s="6" t="n"/>
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
+      <c r="L24" s="6" t="n"/>
+      <c r="M24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
@@ -1265,6 +1424,8 @@
       <c r="I25" s="6" t="n"/>
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6" t="n"/>
+      <c r="M25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
@@ -1281,6 +1442,8 @@
       <c r="I26" s="6" t="n"/>
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n"/>
+      <c r="L26" s="6" t="n"/>
+      <c r="M26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
@@ -1297,6 +1460,8 @@
       <c r="I27" s="6" t="n"/>
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6" t="n"/>
+      <c r="M27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
@@ -1313,6 +1478,8 @@
       <c r="I28" s="6" t="n"/>
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="n"/>
+      <c r="L28" s="6" t="n"/>
+      <c r="M28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
@@ -1329,6 +1496,8 @@
       <c r="I29" s="6" t="n"/>
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n"/>
+      <c r="L29" s="6" t="n"/>
+      <c r="M29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n"/>
@@ -1345,6 +1514,8 @@
       <c r="I30" s="6" t="n"/>
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="n"/>
+      <c r="L30" s="6" t="n"/>
+      <c r="M30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
@@ -1361,6 +1532,8 @@
       <c r="I31" s="6" t="n"/>
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="6" t="n"/>
+      <c r="L31" s="6" t="n"/>
+      <c r="M31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
@@ -1377,6 +1550,8 @@
       <c r="I32" s="6" t="n"/>
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
+      <c r="L32" s="6" t="n"/>
+      <c r="M32" s="6" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:H32">
@@ -1390,7 +1565,7 @@
       <formula>AND(ISNUMBER($H2),$H2&lt;4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="E2:E32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Dominio" error="Puede combinar dos dominios (por ejemplo 'Datos / Procesos'). Pulse Sí para conservar el valor." type="list" errorStyle="warning">
       <formula1>"Negocio,Procesos,Datos,Aplicaciones,Infraestructura,Seguridad,Gobierno TI"</formula1>
     </dataValidation>
@@ -1400,8 +1575,11 @@
     <dataValidation sqref="G2:G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Baja,Media,Alta"</formula1>
     </dataValidation>
+    <dataValidation sqref="M2:M32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Quick win,Corto plazo,Mediano plazo,Largo plazo,Gobernanza / cambios"</formula1>
+    </dataValidation>
     <dataValidation sqref="K2:K32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Quick win,Corto plazo,Mediano plazo,Largo plazo,Gobernanza / cambios"</formula1>
+      <formula1>"Preventivo,Reactivo"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>